<commit_message>
Report: Russian headers, number and date formats
</commit_message>
<xml_diff>
--- a/excel_report/example_report.xlsx
+++ b/excel_report/example_report.xlsx
@@ -19,9 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="DD.MM.YYYY"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -60,10 +61,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,25 +434,25 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>manager</t>
+          <t>Менеджер</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>deals</t>
+          <t>Сделок</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>revenue</t>
+          <t>Выручка</t>
         </is>
       </c>
     </row>
@@ -460,10 +462,10 @@
           <t>Петрова</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>106540</v>
       </c>
     </row>
@@ -473,10 +475,10 @@
           <t>Сидоров</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2" t="n">
         <v>83890</v>
       </c>
     </row>
@@ -486,10 +488,10 @@
           <t>Иванов</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="2" t="n">
         <v>79960</v>
       </c>
     </row>
@@ -508,24 +510,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>product</t>
+          <t>Товар</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>qty</t>
+          <t>Кол-во</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>revenue</t>
+          <t>Выручка</t>
         </is>
       </c>
     </row>
@@ -535,10 +537,10 @@
           <t>Кофемашина</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>151920</v>
       </c>
     </row>
@@ -548,10 +550,10 @@
           <t>Блендер</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2" t="n">
         <v>53910</v>
       </c>
     </row>
@@ -561,10 +563,10 @@
           <t>Чайник</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="2" t="n">
         <v>44820</v>
       </c>
     </row>
@@ -574,10 +576,10 @@
           <t>Тостер</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="2" t="n">
         <v>19740</v>
       </c>
     </row>
@@ -602,12 +604,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>month</t>
+          <t>Месяц</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>revenue</t>
+          <t>Выручка</t>
         </is>
       </c>
     </row>
@@ -617,7 +619,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="2" t="n">
         <v>100550</v>
       </c>
     </row>
@@ -627,7 +629,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>90470</v>
       </c>
     </row>
@@ -637,7 +639,7 @@
           <t>2026-09</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="2" t="n">
         <v>79370</v>
       </c>
     </row>
@@ -656,9 +658,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
   </cols>
@@ -666,37 +668,37 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>Дата</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>manager</t>
+          <t>Менеджер</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>product</t>
+          <t>Товар</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>qty</t>
+          <t>Кол-во</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>Цена</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>revenue</t>
+          <t>Выручка</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>46208</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -709,18 +711,18 @@
           <t>Кофемашина</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
         <v>18990</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="2" t="n">
         <v>37980</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>46209</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -733,18 +735,18 @@
           <t>Чайник</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="2" t="n">
         <v>2490</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="2" t="n">
         <v>12450</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>46215</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -757,18 +759,18 @@
           <t>Блендер</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
         <v>5990</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="2" t="n">
         <v>17970</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>46222</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -781,18 +783,18 @@
           <t>Кофемашина</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="2" t="n">
         <v>18990</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="2" t="n">
         <v>18990</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="3" t="n">
         <v>46228</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -805,18 +807,18 @@
           <t>Тостер</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="2" t="n">
         <v>3290</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="2" t="n">
         <v>13160</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="3" t="n">
         <v>46236</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -829,18 +831,18 @@
           <t>Чайник</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="2" t="n">
         <v>2490</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="2" t="n">
         <v>14940</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="3" t="n">
         <v>46242</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -853,18 +855,18 @@
           <t>Тостер</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="2" t="n">
         <v>3290</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="2" t="n">
         <v>6580</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="3" t="n">
         <v>46249</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -877,18 +879,18 @@
           <t>Кофемашина</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="2" t="n">
         <v>18990</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="2" t="n">
         <v>56970</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="3" t="n">
         <v>46255</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -901,18 +903,18 @@
           <t>Блендер</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="2" t="n">
         <v>5990</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="2" t="n">
         <v>11980</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="3" t="n">
         <v>46268</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -925,18 +927,18 @@
           <t>Чайник</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="2" t="n">
         <v>2490</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="2" t="n">
         <v>17430</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="3" t="n">
         <v>46275</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -949,18 +951,18 @@
           <t>Блендер</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="2" t="n">
         <v>5990</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="2" t="n">
         <v>23960</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="3" t="n">
         <v>46283</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -973,13 +975,13 @@
           <t>Кофемашина</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="2" t="n">
         <v>18990</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="2" t="n">
         <v>37980</v>
       </c>
     </row>

</xml_diff>